<commit_message>
Document Digicon Stop/Approach/Clear as R-Y-G on increasing LCOS ports.
Field wiring is Stop then Approach then Clear; the old docs had Stop and Clear reversed. Also record Signal Manager Main/Diverged and OR Stop/Approach per disc.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/cats/data/LCOS_Layout_Inventory_v85_signal_ports.xlsx
+++ b/cats/data/LCOS_Layout_Inventory_v85_signal_ports.xlsx
@@ -591,7 +591,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Head 6LB T G</t>
+          <t>Head 6LB T R</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -611,7 +611,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -621,7 +621,7 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp G; was S3-6 G/Y/R</t>
+          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp R; was S3-6 R/Y/G</t>
         </is>
       </c>
     </row>
@@ -693,7 +693,7 @@
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp Y; was S3-6 G/Y/R</t>
+          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp Y; was S3-6 R/Y/G</t>
         </is>
       </c>
     </row>
@@ -735,7 +735,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Head 6LB T R</t>
+          <t>Head 6LB T G</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -755,7 +755,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -765,7 +765,7 @@
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp R; was S3-6 G/Y/R</t>
+          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp G; was S3-6 R/Y/G</t>
         </is>
       </c>
     </row>
@@ -807,7 +807,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Head 6LB B G</t>
+          <t>Head 6LB B R</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -827,7 +827,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -837,7 +837,7 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp G; was with 6LB T on OU2</t>
+          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp R; was with 6LB T on OU2</t>
         </is>
       </c>
     </row>
@@ -951,7 +951,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Head 6LB B R</t>
+          <t>Head 6LB B G</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -971,7 +971,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -981,7 +981,7 @@
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp R; was with 6LB T on OU2</t>
+          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp G; was with 6LB T on OU2</t>
         </is>
       </c>
     </row>
@@ -1023,7 +1023,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Head 6LA G</t>
+          <t>Head 6LA R</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1043,7 +1043,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1053,7 +1053,7 @@
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp G; was G on Plane OU2; Y/R on 2L OU3 (OU2-8 is BS cal)</t>
+          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp R; was R on Plane OU2; Y/G on 2L OU3 (OU2-8 is BS cal)</t>
         </is>
       </c>
     </row>
@@ -1125,7 +1125,7 @@
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp Y; was G on Plane OU2; Y/R on 2L OU3 (OU2-8 is BS cal)</t>
+          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp Y; was R on Plane OU2; Y/G on 2L OU3 (OU2-8 is BS cal)</t>
         </is>
       </c>
     </row>
@@ -1167,7 +1167,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Head 6LA R</t>
+          <t>Head 6LA G</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1187,7 +1187,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1197,7 +1197,7 @@
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp R; was G on Plane OU2; Y/R on 2L OU3 (OU2-8 is BS cal)</t>
+          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp G; was R on Plane OU2; Y/G on 2L OU3 (OU2-8 is BS cal)</t>
         </is>
       </c>
     </row>
@@ -1239,7 +1239,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Head 2L T G</t>
+          <t>Head 2L T R</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1259,7 +1259,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1269,7 +1269,7 @@
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>LCOS Signal 6 UID 38; STOP/APPROACH/CLEAR; lamp G; was S3-8 G/Y/R</t>
+          <t>LCOS Signal 6 UID 38; STOP/APPROACH/CLEAR; lamp R; was S3-8 R/Y/G</t>
         </is>
       </c>
     </row>
@@ -1341,7 +1341,7 @@
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>LCOS Signal 6 UID 38; STOP/APPROACH/CLEAR; lamp Y; was S3-8 G/Y/R</t>
+          <t>LCOS Signal 6 UID 38; STOP/APPROACH/CLEAR; lamp Y; was S3-8 R/Y/G</t>
         </is>
       </c>
     </row>
@@ -1383,7 +1383,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Head 2L T R</t>
+          <t>Head 2L T G</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1403,7 +1403,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1413,7 +1413,7 @@
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>LCOS Signal 6 UID 38; STOP/APPROACH/CLEAR; lamp R; was S3-8 G/Y/R</t>
+          <t>LCOS Signal 6 UID 38; STOP/APPROACH/CLEAR; lamp G; was S3-8 R/Y/G</t>
         </is>
       </c>
     </row>
@@ -1455,7 +1455,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Head 2L B G</t>
+          <t>Head 2L B R</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1475,7 +1475,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -1485,7 +1485,7 @@
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>LCOS Signal 7 UID 39; STOP/APPROACH/CLEAR; lamp G; was with 2L T on OU3</t>
+          <t>LCOS Signal 7 UID 39; STOP/APPROACH/CLEAR; lamp R; was with 2L T on OU3</t>
         </is>
       </c>
     </row>
@@ -1599,7 +1599,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Head 2L B R</t>
+          <t>Head 2L B G</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1619,7 +1619,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -1629,7 +1629,7 @@
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>LCOS Signal 7 UID 39; STOP/APPROACH/CLEAR; lamp R; was with 2L T on OU3</t>
+          <t>LCOS Signal 7 UID 39; STOP/APPROACH/CLEAR; lamp G; was with 2L T on OU3</t>
         </is>
       </c>
     </row>
@@ -1671,7 +1671,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Head 4RA G</t>
+          <t>Head 4RA R</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1691,7 +1691,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -1701,7 +1701,7 @@
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp G; was Brick west OU4 with 4RB</t>
+          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp R; was Brick west OU4 with 4RB</t>
         </is>
       </c>
     </row>
@@ -1815,7 +1815,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Head 4RA R</t>
+          <t>Head 4RA G</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1835,7 +1835,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -1845,7 +1845,7 @@
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp R; was Brick west OU4 with 4RB</t>
+          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp G; was Brick west OU4 with 4RB</t>
         </is>
       </c>
     </row>
@@ -1887,7 +1887,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Head 4RB G</t>
+          <t>Head 4RB R</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1907,7 +1907,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -1917,7 +1917,7 @@
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>LCOS Signal 5 UID 37; STOP/APPROACH/CLEAR; lamp G; was Brick west OU4 with 4RA</t>
+          <t>LCOS Signal 5 UID 37; STOP/APPROACH/CLEAR; lamp R; was Brick west OU4 with 4RA</t>
         </is>
       </c>
     </row>
@@ -2031,7 +2031,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Head 4RB R</t>
+          <t>Head 4RB G</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -2051,7 +2051,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -2061,7 +2061,7 @@
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>LCOS Signal 5 UID 37; STOP/APPROACH/CLEAR; lamp R; was Brick west OU4 with 4RA</t>
+          <t>LCOS Signal 5 UID 37; STOP/APPROACH/CLEAR; lamp G; was Brick west OU4 with 4RA</t>
         </is>
       </c>
     </row>
@@ -2103,7 +2103,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Head 8RA T G</t>
+          <t>Head 8RA T R</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -2123,7 +2123,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -2133,7 +2133,7 @@
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp G; was S3-10 G/Y/R</t>
+          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp R; was S3-10 R/Y/G</t>
         </is>
       </c>
     </row>
@@ -2205,7 +2205,7 @@
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp Y; was S3-10 G/Y/R</t>
+          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp Y; was S3-10 R/Y/G</t>
         </is>
       </c>
     </row>
@@ -2247,7 +2247,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Head 8RA T R</t>
+          <t>Head 8RA T G</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -2267,7 +2267,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -2277,7 +2277,7 @@
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp R; was S3-10 G/Y/R</t>
+          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp G; was S3-10 R/Y/G</t>
         </is>
       </c>
     </row>
@@ -2319,7 +2319,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Head 8RA B G</t>
+          <t>Head 8RA B R</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -2339,7 +2339,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -2349,7 +2349,7 @@
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp G; was with 8RA T on OU1</t>
+          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp R; was with 8RA T on OU1</t>
         </is>
       </c>
     </row>
@@ -2463,7 +2463,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Head 8RA B R</t>
+          <t>Head 8RA B G</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -2493,7 +2493,7 @@
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp R; was with 8RA T on OU1</t>
+          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp G; was with 8RA T on OU1</t>
         </is>
       </c>
     </row>
@@ -2535,7 +2535,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Head 8RB T G</t>
+          <t>Head 8RB T R</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -2555,7 +2555,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -2565,7 +2565,7 @@
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>LCOS Signal 3 UID 35; STOP/APPROACH/CLEAR; lamp G; was S3-12; sequential G/Y/R</t>
+          <t>LCOS Signal 3 UID 35; STOP/APPROACH/CLEAR; lamp R; was S3-12; sequential R/Y/G</t>
         </is>
       </c>
     </row>
@@ -2637,7 +2637,7 @@
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>LCOS Signal 3 UID 35; STOP/APPROACH/CLEAR; lamp Y; was S3-12; sequential G/Y/R</t>
+          <t>LCOS Signal 3 UID 35; STOP/APPROACH/CLEAR; lamp Y; was S3-12; sequential R/Y/G</t>
         </is>
       </c>
     </row>
@@ -2679,7 +2679,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Head 8RB T R</t>
+          <t>Head 8RB T G</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -2699,7 +2699,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -2709,7 +2709,7 @@
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>LCOS Signal 3 UID 35; STOP/APPROACH/CLEAR; lamp R; was S3-12; sequential G/Y/R</t>
+          <t>LCOS Signal 3 UID 35; STOP/APPROACH/CLEAR; lamp G; was S3-12; sequential R/Y/G</t>
         </is>
       </c>
     </row>
@@ -2751,7 +2751,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Head 8RB B G</t>
+          <t>Head 8RB B R</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -2771,7 +2771,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -2781,7 +2781,7 @@
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp G; was with 8RB T on OU4</t>
+          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp R; was with 8RB T on OU4</t>
         </is>
       </c>
     </row>
@@ -2895,7 +2895,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Head 8RB B R</t>
+          <t>Head 8RB B G</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -2915,7 +2915,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -2925,7 +2925,7 @@
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp R; was with 8RB T on OU4</t>
+          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp G; was with 8RB T on OU4</t>
         </is>
       </c>
     </row>
@@ -2967,7 +2967,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Head 8LA T G</t>
+          <t>Head 8LA T R</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -2987,7 +2987,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -2997,7 +2997,7 @@
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>LCOS Signal 5 UID 37; STOP/APPROACH/CLEAR; lamp G; was S3-5 G/Y/R</t>
+          <t>LCOS Signal 5 UID 37; STOP/APPROACH/CLEAR; lamp R; was S3-5 R/Y/G</t>
         </is>
       </c>
     </row>
@@ -3069,7 +3069,7 @@
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>LCOS Signal 5 UID 37; STOP/APPROACH/CLEAR; lamp Y; was S3-5 G/Y/R</t>
+          <t>LCOS Signal 5 UID 37; STOP/APPROACH/CLEAR; lamp Y; was S3-5 R/Y/G</t>
         </is>
       </c>
     </row>
@@ -3111,7 +3111,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Head 8LA T R</t>
+          <t>Head 8LA T G</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -3131,7 +3131,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -3141,7 +3141,7 @@
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>LCOS Signal 5 UID 37; STOP/APPROACH/CLEAR; lamp R; was S3-5 G/Y/R</t>
+          <t>LCOS Signal 5 UID 37; STOP/APPROACH/CLEAR; lamp G; was S3-5 R/Y/G</t>
         </is>
       </c>
     </row>
@@ -3183,7 +3183,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Head 8LA B G</t>
+          <t>Head 8LA B R</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -3203,7 +3203,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -3213,7 +3213,7 @@
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>LCOS Signal 6 UID 38; STOP/APPROACH/CLEAR; lamp G; was with 8LA T on OU2</t>
+          <t>LCOS Signal 6 UID 38; STOP/APPROACH/CLEAR; lamp R; was with 8LA T on OU2</t>
         </is>
       </c>
     </row>
@@ -3327,7 +3327,7 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Head 8LA B R</t>
+          <t>Head 8LA B G</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -3347,7 +3347,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
@@ -3357,7 +3357,7 @@
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>LCOS Signal 6 UID 38; STOP/APPROACH/CLEAR; lamp R; was with 8LA T on OU2</t>
+          <t>LCOS Signal 6 UID 38; STOP/APPROACH/CLEAR; lamp G; was with 8LA T on OU2</t>
         </is>
       </c>
     </row>
@@ -3399,7 +3399,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Head 8LB G</t>
+          <t>Head 8LB R</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -3419,7 +3419,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
@@ -3429,7 +3429,7 @@
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp G; was G/Y with 8LA; R spills to 8RB OU4</t>
+          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp R; was R/Y with 8LA; G spills to 8RB OU4</t>
         </is>
       </c>
     </row>
@@ -3501,7 +3501,7 @@
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp Y; was G/Y with 8LA; R spills to 8RB OU4</t>
+          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp Y; was R/Y with 8LA; G spills to 8RB OU4</t>
         </is>
       </c>
     </row>
@@ -3543,7 +3543,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Head 8LB R</t>
+          <t>Head 8LB G</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -3563,7 +3563,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
@@ -3573,7 +3573,7 @@
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp R; was G/Y with 8LA; R spills to 8RB OU4</t>
+          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp G; was R/Y with 8LA; G spills to 8RB OU4</t>
         </is>
       </c>
     </row>
@@ -3615,7 +3615,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>Head 24RA T G</t>
+          <t>Head 24RA T R</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -3635,7 +3635,7 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
@@ -3645,7 +3645,7 @@
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp G; was C2-OU1 5V</t>
+          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp R; was C2-OU1 5V</t>
         </is>
       </c>
     </row>
@@ -3759,7 +3759,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>Head 24RA T R</t>
+          <t>Head 24RA T G</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -3779,7 +3779,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
@@ -3789,7 +3789,7 @@
       </c>
       <c r="N47" t="inlineStr">
         <is>
-          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp R; was C2-OU1 5V</t>
+          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp G; was C2-OU1 5V</t>
         </is>
       </c>
     </row>
@@ -3831,7 +3831,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>Head 24RA B G</t>
+          <t>Head 24RA B R</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -3851,7 +3851,7 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
@@ -3861,7 +3861,7 @@
       </c>
       <c r="N48" t="inlineStr">
         <is>
-          <t>LCOS Signal 6 UID 38; STOP/APPROACH/CLEAR; lamp G; was with 24RA T on OU1</t>
+          <t>LCOS Signal 6 UID 38; STOP/APPROACH/CLEAR; lamp R; was with 24RA T on OU1</t>
         </is>
       </c>
     </row>
@@ -3975,7 +3975,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>Head 24RA B R</t>
+          <t>Head 24RA B G</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
@@ -3995,7 +3995,7 @@
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M50" t="inlineStr">
@@ -4005,7 +4005,7 @@
       </c>
       <c r="N50" t="inlineStr">
         <is>
-          <t>LCOS Signal 6 UID 38; STOP/APPROACH/CLEAR; lamp R; was with 24RA T on OU1</t>
+          <t>LCOS Signal 6 UID 38; STOP/APPROACH/CLEAR; lamp G; was with 24RA T on OU1</t>
         </is>
       </c>
     </row>
@@ -4047,7 +4047,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>Head 24RB G</t>
+          <t>Head 24RB R</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -4067,7 +4067,7 @@
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M51" t="inlineStr">
@@ -4077,7 +4077,7 @@
       </c>
       <c r="N51" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp G; was whole dwarf on leftover OU3 (OU1-8 is BS cal)</t>
+          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp R; was whole dwarf on leftover OU3 (OU1-8 is BS cal)</t>
         </is>
       </c>
     </row>
@@ -4191,7 +4191,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>Head 24RB R</t>
+          <t>Head 24RB G</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
@@ -4211,7 +4211,7 @@
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M53" t="inlineStr">
@@ -4221,7 +4221,7 @@
       </c>
       <c r="N53" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp R; was whole dwarf on leftover OU3 (OU1-8 is BS cal)</t>
+          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp G; was whole dwarf on leftover OU3 (OU1-8 is BS cal)</t>
         </is>
       </c>
     </row>
@@ -4263,7 +4263,7 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>Head 24L T G</t>
+          <t>Head 24L T R</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
@@ -4283,7 +4283,7 @@
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M54" t="inlineStr">
@@ -4293,7 +4293,7 @@
       </c>
       <c r="N54" t="inlineStr">
         <is>
-          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp G; was with 24RA cluster</t>
+          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp R; was with 24RA cluster</t>
         </is>
       </c>
     </row>
@@ -4407,7 +4407,7 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>Head 24L T R</t>
+          <t>Head 24L T G</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -4427,7 +4427,7 @@
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M56" t="inlineStr">
@@ -4437,7 +4437,7 @@
       </c>
       <c r="N56" t="inlineStr">
         <is>
-          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp R; was with 24RA cluster</t>
+          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp G; was with 24RA cluster</t>
         </is>
       </c>
     </row>
@@ -4479,7 +4479,7 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>Head 24L B G</t>
+          <t>Head 24L B R</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -4499,7 +4499,7 @@
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M57" t="inlineStr">
@@ -4509,7 +4509,7 @@
       </c>
       <c r="N57" t="inlineStr">
         <is>
-          <t>LCOS Signal 7 UID 39; STOP/APPROACH/CLEAR; lamp G; was with 24L T on OU2</t>
+          <t>LCOS Signal 7 UID 39; STOP/APPROACH/CLEAR; lamp R; was with 24L T on OU2</t>
         </is>
       </c>
     </row>
@@ -4623,7 +4623,7 @@
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>Head 24L B R</t>
+          <t>Head 24L B G</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -4643,7 +4643,7 @@
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M59" t="inlineStr">
@@ -4653,7 +4653,7 @@
       </c>
       <c r="N59" t="inlineStr">
         <is>
-          <t>LCOS Signal 7 UID 39; STOP/APPROACH/CLEAR; lamp R; was with 24L T on OU2</t>
+          <t>LCOS Signal 7 UID 39; STOP/APPROACH/CLEAR; lamp G; was with 24L T on OU2</t>
         </is>
       </c>
     </row>
@@ -4695,7 +4695,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>Head 34L T G</t>
+          <t>Head 34L T R</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -4715,7 +4715,7 @@
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M60" t="inlineStr">
@@ -4725,7 +4725,7 @@
       </c>
       <c r="N60" t="inlineStr">
         <is>
-          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp G; was was C2 235</t>
+          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp R; was was C2 235</t>
         </is>
       </c>
     </row>
@@ -4839,7 +4839,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>Head 34L T R</t>
+          <t>Head 34L T G</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -4859,7 +4859,7 @@
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M62" t="inlineStr">
@@ -4869,7 +4869,7 @@
       </c>
       <c r="N62" t="inlineStr">
         <is>
-          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp R; was was C2 235</t>
+          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp G; was was C2 235</t>
         </is>
       </c>
     </row>
@@ -4911,7 +4911,7 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>Head 34L B G</t>
+          <t>Head 34L B R</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -4931,7 +4931,7 @@
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M63" t="inlineStr">
@@ -4941,7 +4941,7 @@
       </c>
       <c r="N63" t="inlineStr">
         <is>
-          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp G; was with 34L T on OU2</t>
+          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp R; was with 34L T on OU2</t>
         </is>
       </c>
     </row>
@@ -5055,7 +5055,7 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>Head 34L B R</t>
+          <t>Head 34L B G</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -5075,7 +5075,7 @@
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M65" t="inlineStr">
@@ -5085,7 +5085,7 @@
       </c>
       <c r="N65" t="inlineStr">
         <is>
-          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp R; was with 34L T on OU2</t>
+          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp G; was with 34L T on OU2</t>
         </is>
       </c>
     </row>
@@ -5127,7 +5127,7 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>Head 32R G</t>
+          <t>Head 32R R</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -5147,7 +5147,7 @@
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M66" t="inlineStr">
@@ -5157,7 +5157,7 @@
       </c>
       <c r="N66" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp G; was G with 34L; Y/R on 34R OU3 (OU2-8 is BS cal)</t>
+          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp R; was R with 34L; Y/G on 34R OU3 (OU2-8 is BS cal)</t>
         </is>
       </c>
     </row>
@@ -5229,7 +5229,7 @@
       </c>
       <c r="N67" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp Y; was G with 34L; Y/R on 34R OU3 (OU2-8 is BS cal)</t>
+          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp Y; was R with 34L; Y/G on 34R OU3 (OU2-8 is BS cal)</t>
         </is>
       </c>
     </row>
@@ -5271,7 +5271,7 @@
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>Head 32R R</t>
+          <t>Head 32R G</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -5291,7 +5291,7 @@
       </c>
       <c r="L68" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M68" t="inlineStr">
@@ -5301,7 +5301,7 @@
       </c>
       <c r="N68" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp R; was G with 34L; Y/R on 34R OU3 (OU2-8 is BS cal)</t>
+          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp G; was R with 34L; Y/G on 34R OU3 (OU2-8 is BS cal)</t>
         </is>
       </c>
     </row>
@@ -5343,7 +5343,7 @@
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>Head 34R T G</t>
+          <t>Head 34R T R</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -5363,7 +5363,7 @@
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M69" t="inlineStr">
@@ -5373,7 +5373,7 @@
       </c>
       <c r="N69" t="inlineStr">
         <is>
-          <t>LCOS Signal 3 UID 35; STOP/APPROACH/CLEAR; lamp G; was was C2 237</t>
+          <t>LCOS Signal 3 UID 35; STOP/APPROACH/CLEAR; lamp R; was was C2 237</t>
         </is>
       </c>
     </row>
@@ -5487,7 +5487,7 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>Head 34R T R</t>
+          <t>Head 34R T G</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -5507,7 +5507,7 @@
       </c>
       <c r="L71" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M71" t="inlineStr">
@@ -5517,7 +5517,7 @@
       </c>
       <c r="N71" t="inlineStr">
         <is>
-          <t>LCOS Signal 3 UID 35; STOP/APPROACH/CLEAR; lamp R; was was C2 237</t>
+          <t>LCOS Signal 3 UID 35; STOP/APPROACH/CLEAR; lamp G; was was C2 237</t>
         </is>
       </c>
     </row>
@@ -5559,7 +5559,7 @@
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>Head 34R B G</t>
+          <t>Head 34R B R</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -5579,7 +5579,7 @@
       </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M72" t="inlineStr">
@@ -5589,7 +5589,7 @@
       </c>
       <c r="N72" t="inlineStr">
         <is>
-          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp G; was with 34R T on OU3</t>
+          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp R; was with 34R T on OU3</t>
         </is>
       </c>
     </row>
@@ -5703,7 +5703,7 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>Head 34R B R</t>
+          <t>Head 34R B G</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
@@ -5723,7 +5723,7 @@
       </c>
       <c r="L74" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M74" t="inlineStr">
@@ -5733,7 +5733,7 @@
       </c>
       <c r="N74" t="inlineStr">
         <is>
-          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp R; was with 34R T on OU3</t>
+          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp G; was with 34R T on OU3</t>
         </is>
       </c>
     </row>
@@ -5775,7 +5775,7 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>Head 36RA T G</t>
+          <t>Head 36RA T R</t>
         </is>
       </c>
       <c r="I75" t="inlineStr">
@@ -5795,7 +5795,7 @@
       </c>
       <c r="L75" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M75" t="inlineStr">
@@ -5805,7 +5805,7 @@
       </c>
       <c r="N75" t="inlineStr">
         <is>
-          <t>LCOS Signal 3 UID 35; STOP/APPROACH/CLEAR; lamp G; was S1-2 G/Y/R</t>
+          <t>LCOS Signal 3 UID 35; STOP/APPROACH/CLEAR; lamp R; was S1-2 R/Y/G</t>
         </is>
       </c>
     </row>
@@ -5877,7 +5877,7 @@
       </c>
       <c r="N76" t="inlineStr">
         <is>
-          <t>LCOS Signal 3 UID 35; STOP/APPROACH/CLEAR; lamp Y; was S1-2 G/Y/R</t>
+          <t>LCOS Signal 3 UID 35; STOP/APPROACH/CLEAR; lamp Y; was S1-2 R/Y/G</t>
         </is>
       </c>
     </row>
@@ -5919,7 +5919,7 @@
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>Head 36RA T R</t>
+          <t>Head 36RA T G</t>
         </is>
       </c>
       <c r="I77" t="inlineStr">
@@ -5939,7 +5939,7 @@
       </c>
       <c r="L77" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M77" t="inlineStr">
@@ -5949,7 +5949,7 @@
       </c>
       <c r="N77" t="inlineStr">
         <is>
-          <t>LCOS Signal 3 UID 35; STOP/APPROACH/CLEAR; lamp R; was S1-2 G/Y/R</t>
+          <t>LCOS Signal 3 UID 35; STOP/APPROACH/CLEAR; lamp G; was S1-2 R/Y/G</t>
         </is>
       </c>
     </row>
@@ -5991,7 +5991,7 @@
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>Head 36RA B G</t>
+          <t>Head 36RA B R</t>
         </is>
       </c>
       <c r="I78" t="inlineStr">
@@ -6011,7 +6011,7 @@
       </c>
       <c r="L78" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M78" t="inlineStr">
@@ -6021,7 +6021,7 @@
       </c>
       <c r="N78" t="inlineStr">
         <is>
-          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp G; was with 36RA T on OU2</t>
+          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp R; was with 36RA T on OU2</t>
         </is>
       </c>
     </row>
@@ -6135,7 +6135,7 @@
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>Head 36RA B R</t>
+          <t>Head 36RA B G</t>
         </is>
       </c>
       <c r="I80" t="inlineStr">
@@ -6155,7 +6155,7 @@
       </c>
       <c r="L80" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M80" t="inlineStr">
@@ -6165,7 +6165,7 @@
       </c>
       <c r="N80" t="inlineStr">
         <is>
-          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp R; was with 36RA T on OU2</t>
+          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp G; was with 36RA T on OU2</t>
         </is>
       </c>
     </row>
@@ -6207,7 +6207,7 @@
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>Head 36RB T G</t>
+          <t>Head 36RB T R</t>
         </is>
       </c>
       <c r="I81" t="inlineStr">
@@ -6227,7 +6227,7 @@
       </c>
       <c r="L81" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M81" t="inlineStr">
@@ -6237,7 +6237,7 @@
       </c>
       <c r="N81" t="inlineStr">
         <is>
-          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp G; was was C11 1132</t>
+          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp R; was was C11 1132</t>
         </is>
       </c>
     </row>
@@ -6351,7 +6351,7 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>Head 36RB T R</t>
+          <t>Head 36RB T G</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -6371,7 +6371,7 @@
       </c>
       <c r="L83" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M83" t="inlineStr">
@@ -6381,7 +6381,7 @@
       </c>
       <c r="N83" t="inlineStr">
         <is>
-          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp R; was was C11 1132</t>
+          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp G; was was C11 1132</t>
         </is>
       </c>
     </row>
@@ -6423,7 +6423,7 @@
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>Head 36RB B G</t>
+          <t>Head 36RB B R</t>
         </is>
       </c>
       <c r="I84" t="inlineStr">
@@ -6443,7 +6443,7 @@
       </c>
       <c r="L84" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M84" t="inlineStr">
@@ -6453,7 +6453,7 @@
       </c>
       <c r="N84" t="inlineStr">
         <is>
-          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp G; was with 36RB T on OU3</t>
+          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp R; was with 36RB T on OU3</t>
         </is>
       </c>
     </row>
@@ -6567,7 +6567,7 @@
       </c>
       <c r="H86" t="inlineStr">
         <is>
-          <t>Head 36RB B R</t>
+          <t>Head 36RB B G</t>
         </is>
       </c>
       <c r="I86" t="inlineStr">
@@ -6587,7 +6587,7 @@
       </c>
       <c r="L86" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M86" t="inlineStr">
@@ -6597,7 +6597,7 @@
       </c>
       <c r="N86" t="inlineStr">
         <is>
-          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp R; was with 36RB T on OU3</t>
+          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp G; was with 36RB T on OU3</t>
         </is>
       </c>
     </row>
@@ -6639,7 +6639,7 @@
       </c>
       <c r="H87" t="inlineStr">
         <is>
-          <t>Head 38LB T G</t>
+          <t>Head 38LB T R</t>
         </is>
       </c>
       <c r="I87" t="inlineStr">
@@ -6659,7 +6659,7 @@
       </c>
       <c r="L87" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M87" t="inlineStr">
@@ -6669,7 +6669,7 @@
       </c>
       <c r="N87" t="inlineStr">
         <is>
-          <t>LCOS Signal 7 UID 39; STOP/APPROACH/CLEAR; lamp G; was S1-3 G/Y/R</t>
+          <t>LCOS Signal 7 UID 39; STOP/APPROACH/CLEAR; lamp R; was S1-3 R/Y/G</t>
         </is>
       </c>
     </row>
@@ -6741,7 +6741,7 @@
       </c>
       <c r="N88" t="inlineStr">
         <is>
-          <t>LCOS Signal 7 UID 39; STOP/APPROACH/CLEAR; lamp Y; was S1-3 G/Y/R</t>
+          <t>LCOS Signal 7 UID 39; STOP/APPROACH/CLEAR; lamp Y; was S1-3 R/Y/G</t>
         </is>
       </c>
     </row>
@@ -6783,7 +6783,7 @@
       </c>
       <c r="H89" t="inlineStr">
         <is>
-          <t>Head 38LB T R</t>
+          <t>Head 38LB T G</t>
         </is>
       </c>
       <c r="I89" t="inlineStr">
@@ -6803,7 +6803,7 @@
       </c>
       <c r="L89" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M89" t="inlineStr">
@@ -6813,7 +6813,7 @@
       </c>
       <c r="N89" t="inlineStr">
         <is>
-          <t>LCOS Signal 7 UID 39; STOP/APPROACH/CLEAR; lamp R; was S1-3 G/Y/R</t>
+          <t>LCOS Signal 7 UID 39; STOP/APPROACH/CLEAR; lamp G; was S1-3 R/Y/G</t>
         </is>
       </c>
     </row>
@@ -6855,7 +6855,7 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>Head 38LB B G</t>
+          <t>Head 38LB B R</t>
         </is>
       </c>
       <c r="I90" t="inlineStr">
@@ -6875,7 +6875,7 @@
       </c>
       <c r="L90" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M90" t="inlineStr">
@@ -6885,7 +6885,7 @@
       </c>
       <c r="N90" t="inlineStr">
         <is>
-          <t>LCOS Signal 8 UID 40; STOP/APPROACH/CLEAR; lamp G; was with 38LB T on OU4</t>
+          <t>LCOS Signal 8 UID 40; STOP/APPROACH/CLEAR; lamp R; was with 38LB T on OU4</t>
         </is>
       </c>
     </row>
@@ -6999,7 +6999,7 @@
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>Head 38LB B R</t>
+          <t>Head 38LB B G</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
@@ -7019,7 +7019,7 @@
       </c>
       <c r="L92" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M92" t="inlineStr">
@@ -7029,7 +7029,7 @@
       </c>
       <c r="N92" t="inlineStr">
         <is>
-          <t>LCOS Signal 8 UID 40; STOP/APPROACH/CLEAR; lamp R; was with 38LB T on OU4</t>
+          <t>LCOS Signal 8 UID 40; STOP/APPROACH/CLEAR; lamp G; was with 38LB T on OU4</t>
         </is>
       </c>
     </row>
@@ -7071,7 +7071,7 @@
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>Head 38LA G</t>
+          <t>Head 38LA R</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
@@ -7091,7 +7091,7 @@
       </c>
       <c r="L93" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M93" t="inlineStr">
@@ -7101,7 +7101,7 @@
       </c>
       <c r="N93" t="inlineStr">
         <is>
-          <t>LCOS Signal 11 UID 43; STOP/APPROACH/CLEAR; lamp G; was leftover trio on 36 boards; 38LB keeps OU4</t>
+          <t>LCOS Signal 11 UID 43; STOP/APPROACH/CLEAR; lamp R; was leftover trio on 36 boards; 38LB keeps OU4</t>
         </is>
       </c>
     </row>
@@ -7215,7 +7215,7 @@
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>Head 38LA R</t>
+          <t>Head 38LA G</t>
         </is>
       </c>
       <c r="I95" t="inlineStr">
@@ -7235,7 +7235,7 @@
       </c>
       <c r="L95" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M95" t="inlineStr">
@@ -7245,7 +7245,7 @@
       </c>
       <c r="N95" t="inlineStr">
         <is>
-          <t>LCOS Signal 11 UID 43; STOP/APPROACH/CLEAR; lamp R; was leftover trio on 36 boards; 38LB keeps OU4</t>
+          <t>LCOS Signal 11 UID 43; STOP/APPROACH/CLEAR; lamp G; was leftover trio on 36 boards; 38LB keeps OU4</t>
         </is>
       </c>
     </row>
@@ -7287,7 +7287,7 @@
       </c>
       <c r="H96" t="inlineStr">
         <is>
-          <t>Head 40LB T G</t>
+          <t>Head 40LB T R</t>
         </is>
       </c>
       <c r="I96" t="inlineStr">
@@ -7307,7 +7307,7 @@
       </c>
       <c r="L96" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M96" t="inlineStr">
@@ -7317,7 +7317,7 @@
       </c>
       <c r="N96" t="inlineStr">
         <is>
-          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp G; was was C1 132</t>
+          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp R; was was C1 132</t>
         </is>
       </c>
     </row>
@@ -7431,7 +7431,7 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>Head 40LB T R</t>
+          <t>Head 40LB T G</t>
         </is>
       </c>
       <c r="I98" t="inlineStr">
@@ -7451,7 +7451,7 @@
       </c>
       <c r="L98" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M98" t="inlineStr">
@@ -7461,7 +7461,7 @@
       </c>
       <c r="N98" t="inlineStr">
         <is>
-          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp R; was was C1 132</t>
+          <t>LCOS Signal 0 UID 32; STOP/APPROACH/CLEAR; lamp G; was was C1 132</t>
         </is>
       </c>
     </row>
@@ -7503,7 +7503,7 @@
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>Head 40LB B G</t>
+          <t>Head 40LB B R</t>
         </is>
       </c>
       <c r="I99" t="inlineStr">
@@ -7523,7 +7523,7 @@
       </c>
       <c r="L99" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M99" t="inlineStr">
@@ -7533,7 +7533,7 @@
       </c>
       <c r="N99" t="inlineStr">
         <is>
-          <t>LCOS Signal 3 UID 35; STOP/APPROACH/CLEAR; lamp G; was with 40LB T on OU2</t>
+          <t>LCOS Signal 3 UID 35; STOP/APPROACH/CLEAR; lamp R; was with 40LB T on OU2</t>
         </is>
       </c>
     </row>
@@ -7647,7 +7647,7 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>Head 40LB B R</t>
+          <t>Head 40LB B G</t>
         </is>
       </c>
       <c r="I101" t="inlineStr">
@@ -7667,7 +7667,7 @@
       </c>
       <c r="L101" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M101" t="inlineStr">
@@ -7677,7 +7677,7 @@
       </c>
       <c r="N101" t="inlineStr">
         <is>
-          <t>LCOS Signal 3 UID 35; STOP/APPROACH/CLEAR; lamp R; was with 40LB T on OU2</t>
+          <t>LCOS Signal 3 UID 35; STOP/APPROACH/CLEAR; lamp G; was with 40LB T on OU2</t>
         </is>
       </c>
     </row>
@@ -7719,7 +7719,7 @@
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>Head 40LA G</t>
+          <t>Head 40LA R</t>
         </is>
       </c>
       <c r="I102" t="inlineStr">
@@ -7739,7 +7739,7 @@
       </c>
       <c r="L102" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M102" t="inlineStr">
@@ -7749,7 +7749,7 @@
       </c>
       <c r="N102" t="inlineStr">
         <is>
-          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp G; was whole dwarf on OU3; 2035/2036 can sit apart</t>
+          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp R; was whole dwarf on OU3; 2035/2036 can sit apart</t>
         </is>
       </c>
     </row>
@@ -7863,7 +7863,7 @@
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>Head 40LA R</t>
+          <t>Head 40LA G</t>
         </is>
       </c>
       <c r="I104" t="inlineStr">
@@ -7883,7 +7883,7 @@
       </c>
       <c r="L104" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M104" t="inlineStr">
@@ -7893,7 +7893,7 @@
       </c>
       <c r="N104" t="inlineStr">
         <is>
-          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp R; was whole dwarf on OU3; 2035/2036 can sit apart</t>
+          <t>LCOS Signal 4 UID 36; STOP/APPROACH/CLEAR; lamp G; was whole dwarf on OU3; 2035/2036 can sit apart</t>
         </is>
       </c>
     </row>
@@ -7935,7 +7935,7 @@
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>Head 2036 G</t>
+          <t>Head 2036 R</t>
         </is>
       </c>
       <c r="I105" t="inlineStr">
@@ -7955,7 +7955,7 @@
       </c>
       <c r="L105" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M105" t="inlineStr">
@@ -7965,7 +7965,7 @@
       </c>
       <c r="N105" t="inlineStr">
         <is>
-          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp G; was balloon; sequential G/Y/R</t>
+          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp R; was balloon; sequential R/Y/G</t>
         </is>
       </c>
     </row>
@@ -8037,7 +8037,7 @@
       </c>
       <c r="N106" t="inlineStr">
         <is>
-          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp Y; was balloon; sequential G/Y/R</t>
+          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp Y; was balloon; sequential R/Y/G</t>
         </is>
       </c>
     </row>
@@ -8079,7 +8079,7 @@
       </c>
       <c r="H107" t="inlineStr">
         <is>
-          <t>Head 2036 R</t>
+          <t>Head 2036 G</t>
         </is>
       </c>
       <c r="I107" t="inlineStr">
@@ -8099,7 +8099,7 @@
       </c>
       <c r="L107" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M107" t="inlineStr">
@@ -8109,7 +8109,7 @@
       </c>
       <c r="N107" t="inlineStr">
         <is>
-          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp R; was balloon; sequential G/Y/R</t>
+          <t>LCOS Signal 1 UID 33; STOP/APPROACH/CLEAR; lamp G; was balloon; sequential R/Y/G</t>
         </is>
       </c>
     </row>
@@ -8151,7 +8151,7 @@
       </c>
       <c r="H108" t="inlineStr">
         <is>
-          <t>Head 2035 G</t>
+          <t>Head 2035 R</t>
         </is>
       </c>
       <c r="I108" t="inlineStr">
@@ -8171,7 +8171,7 @@
       </c>
       <c r="L108" t="inlineStr">
         <is>
-          <t>G</t>
+          <t>R</t>
         </is>
       </c>
       <c r="M108" t="inlineStr">
@@ -8181,7 +8181,7 @@
       </c>
       <c r="N108" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp G; was leftover trio (OU2-8 is BS cal)</t>
+          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp R; was leftover trio (OU2-8 is BS cal)</t>
         </is>
       </c>
     </row>
@@ -8295,7 +8295,7 @@
       </c>
       <c r="H110" t="inlineStr">
         <is>
-          <t>Head 2035 R</t>
+          <t>Head 2035 G</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
@@ -8315,7 +8315,7 @@
       </c>
       <c r="L110" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>G</t>
         </is>
       </c>
       <c r="M110" t="inlineStr">
@@ -8325,7 +8325,7 @@
       </c>
       <c r="N110" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp R; was leftover trio (OU2-8 is BS cal)</t>
+          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp G; was leftover trio (OU2-8 is BS cal)</t>
         </is>
       </c>
     </row>
@@ -8411,7 +8411,7 @@
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>SL-2-digicon</t>
+          <t>CO-33-hi</t>
         </is>
       </c>
       <c r="F115" t="inlineStr">
@@ -8421,7 +8421,7 @@
       </c>
       <c r="G115" t="inlineStr">
         <is>
-          <t>IF$shsm:hart-aar:SL-2-digicon(IH432)(IH433)</t>
+          <t>IF$shsm:C&amp;O-1980:CO-33-hi(IH432)(IH433)</t>
         </is>
       </c>
       <c r="H115" t="inlineStr">
@@ -8463,7 +8463,7 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>SL-1-low</t>
+          <t>CO-3-dwarf</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
@@ -8473,7 +8473,7 @@
       </c>
       <c r="G116" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH434)</t>
+          <t>IF$shsm:C&amp;O-1980:CO-3-dwarf(IH434)</t>
         </is>
       </c>
       <c r="H116" t="inlineStr">
@@ -8515,7 +8515,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>SL-2-digicon</t>
+          <t>CO-33-hi</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -8525,7 +8525,7 @@
       </c>
       <c r="G117" t="inlineStr">
         <is>
-          <t>IF$shsm:hart-aar:SL-2-digicon(IH438)(IH439)</t>
+          <t>IF$shsm:C&amp;O-1980:CO-33-hi(IH438)(IH439)</t>
         </is>
       </c>
       <c r="H117" t="inlineStr">
@@ -8567,7 +8567,7 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>SL-1-low</t>
+          <t>CO-3-dwarf</t>
         </is>
       </c>
       <c r="F118" t="inlineStr">
@@ -8577,7 +8577,7 @@
       </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH436)</t>
+          <t>IF$shsm:C&amp;O-1980:CO-3-dwarf(IH436)</t>
         </is>
       </c>
       <c r="H118" t="inlineStr">
@@ -8619,7 +8619,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>SL-1-low</t>
+          <t>CO-3-dwarf</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
@@ -8629,7 +8629,7 @@
       </c>
       <c r="G119" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH437)</t>
+          <t>IF$shsm:C&amp;O-1980:CO-3-dwarf(IH437)</t>
         </is>
       </c>
       <c r="H119" t="inlineStr">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>SL-2-digicon</t>
+          <t>CO-33-hi</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -8681,7 +8681,7 @@
       </c>
       <c r="G120" t="inlineStr">
         <is>
-          <t>IF$shsm:hart-aar:SL-2-digicon(IH1332)(IH1333)</t>
+          <t>IF$shsm:C&amp;O-1980:CO-33-hi(IH1332)(IH1333)</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
@@ -8723,7 +8723,7 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>SL-2-digicon</t>
+          <t>CO-33-hi</t>
         </is>
       </c>
       <c r="F121" t="inlineStr">
@@ -8733,7 +8733,7 @@
       </c>
       <c r="G121" t="inlineStr">
         <is>
-          <t>IF$shsm:hart-aar:SL-2-digicon(IH1335)(IH1336)</t>
+          <t>IF$shsm:C&amp;O-1980:CO-33-hi(IH1335)(IH1336)</t>
         </is>
       </c>
       <c r="H121" t="inlineStr">
@@ -8775,7 +8775,7 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>SL-2-digicon</t>
+          <t>CO-33-hi</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
@@ -8785,7 +8785,7 @@
       </c>
       <c r="G122" t="inlineStr">
         <is>
-          <t>IF$shsm:hart-aar:SL-2-digicon(IH1337)(IH1338)</t>
+          <t>IF$shsm:C&amp;O-1980:CO-33-hi(IH1337)(IH1338)</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
@@ -8827,7 +8827,7 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>SL-1-low</t>
+          <t>CO-3-dwarf</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
@@ -8837,7 +8837,7 @@
       </c>
       <c r="G123" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH1334)</t>
+          <t>IF$shsm:C&amp;O-1980:CO-3-dwarf(IH1334)</t>
         </is>
       </c>
       <c r="H123" t="inlineStr">
@@ -8879,7 +8879,7 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>SL-2-digicon</t>
+          <t>CO-33-hi</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
@@ -8889,7 +8889,7 @@
       </c>
       <c r="G124" t="inlineStr">
         <is>
-          <t>IF$shsm:hart-aar:SL-2-digicon(IH232)(IH238)</t>
+          <t>IF$shsm:C&amp;O-1980:CO-33-hi(IH232)(IH238)</t>
         </is>
       </c>
       <c r="H124" t="inlineStr">
@@ -8931,7 +8931,7 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>SL-1-low</t>
+          <t>CO-3-dwarf</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
@@ -8941,7 +8941,7 @@
       </c>
       <c r="G125" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH234)</t>
+          <t>IF$shsm:C&amp;O-1980:CO-3-dwarf(IH234)</t>
         </is>
       </c>
       <c r="H125" t="inlineStr">
@@ -8983,7 +8983,7 @@
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>SL-2-digicon</t>
+          <t>CO-33-hi</t>
         </is>
       </c>
       <c r="F126" t="inlineStr">
@@ -8993,7 +8993,7 @@
       </c>
       <c r="G126" t="inlineStr">
         <is>
-          <t>IF$shsm:hart-aar:SL-2-digicon(IH233)(IH239)</t>
+          <t>IF$shsm:C&amp;O-1980:CO-33-hi(IH233)(IH239)</t>
         </is>
       </c>
       <c r="H126" t="inlineStr">
@@ -9035,7 +9035,7 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>SL-2-digicon</t>
+          <t>CO-33-hi</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
@@ -9045,7 +9045,7 @@
       </c>
       <c r="G127" t="inlineStr">
         <is>
-          <t>IF$shsm:hart-aar:SL-2-digicon(IH1232)(IH1233)</t>
+          <t>IF$shsm:C&amp;O-1980:CO-33-hi(IH1232)(IH1233)</t>
         </is>
       </c>
       <c r="H127" t="inlineStr">
@@ -9087,7 +9087,7 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>SL-1-low</t>
+          <t>CO-3-dwarf</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
@@ -9097,7 +9097,7 @@
       </c>
       <c r="G128" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH1234)</t>
+          <t>IF$shsm:C&amp;O-1980:CO-3-dwarf(IH1234)</t>
         </is>
       </c>
       <c r="H128" t="inlineStr">
@@ -9139,7 +9139,7 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>SL-2-digicon</t>
+          <t>CO-33-hi</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
@@ -9149,7 +9149,7 @@
       </c>
       <c r="G129" t="inlineStr">
         <is>
-          <t>IF$shsm:hart-aar:SL-2-digicon(IH1235)(IH1236)</t>
+          <t>IF$shsm:C&amp;O-1980:CO-33-hi(IH1235)(IH1236)</t>
         </is>
       </c>
       <c r="H129" t="inlineStr">
@@ -9191,7 +9191,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>SL-2-digicon</t>
+          <t>CO-33-hi</t>
         </is>
       </c>
       <c r="F130" t="inlineStr">
@@ -9201,7 +9201,7 @@
       </c>
       <c r="G130" t="inlineStr">
         <is>
-          <t>IF$shsm:hart-aar:SL-2-digicon(IH135)(IH136)</t>
+          <t>IF$shsm:C&amp;O-1980:CO-33-hi(IH135)(IH136)</t>
         </is>
       </c>
       <c r="H130" t="inlineStr">
@@ -9243,7 +9243,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>SL-2-digicon</t>
+          <t>CO-33-hi</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
@@ -9253,7 +9253,7 @@
       </c>
       <c r="G131" t="inlineStr">
         <is>
-          <t>IF$shsm:hart-aar:SL-2-digicon(IH132)(IH133)</t>
+          <t>IF$shsm:C&amp;O-1980:CO-33-hi(IH132)(IH133)</t>
         </is>
       </c>
       <c r="H131" t="inlineStr">
@@ -9295,7 +9295,7 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>SL-2-digicon</t>
+          <t>CO-33-hi</t>
         </is>
       </c>
       <c r="F132" t="inlineStr">
@@ -9305,7 +9305,7 @@
       </c>
       <c r="G132" t="inlineStr">
         <is>
-          <t>IF$shsm:hart-aar:SL-2-digicon(IH139)(IH140)</t>
+          <t>IF$shsm:C&amp;O-1980:CO-33-hi(IH139)(IH140)</t>
         </is>
       </c>
       <c r="H132" t="inlineStr">
@@ -9347,7 +9347,7 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>SL-1-low</t>
+          <t>CO-3-dwarf</t>
         </is>
       </c>
       <c r="F133" t="inlineStr">
@@ -9357,7 +9357,7 @@
       </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH143)</t>
+          <t>IF$shsm:C&amp;O-1980:CO-3-dwarf(IH143)</t>
         </is>
       </c>
       <c r="H133" t="inlineStr">
@@ -9399,7 +9399,7 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>SL-2-digicon</t>
+          <t>CO-33-hi</t>
         </is>
       </c>
       <c r="F134" t="inlineStr">
@@ -9409,7 +9409,7 @@
       </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>IF$shsm:hart-aar:SL-2-digicon(IH1132)(IH1135)</t>
+          <t>IF$shsm:C&amp;O-1980:CO-33-hi(IH1132)(IH1135)</t>
         </is>
       </c>
       <c r="H134" t="inlineStr">
@@ -9451,7 +9451,7 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>SL-1-low</t>
+          <t>CO-3-dwarf</t>
         </is>
       </c>
       <c r="F135" t="inlineStr">
@@ -9461,7 +9461,7 @@
       </c>
       <c r="G135" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH1136)</t>
+          <t>IF$shsm:C&amp;O-1980:CO-3-dwarf(IH1136)</t>
         </is>
       </c>
       <c r="H135" t="inlineStr">
@@ -9503,7 +9503,7 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>SL-1-low</t>
+          <t>CO-3-dwarf</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
@@ -9513,7 +9513,7 @@
       </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH1133)</t>
+          <t>IF$shsm:C&amp;O-1980:CO-3-dwarf(IH1133)</t>
         </is>
       </c>
       <c r="H136" t="inlineStr">
@@ -9555,7 +9555,7 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>SL-1-low</t>
+          <t>CO-3-dwarf</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
@@ -9565,7 +9565,7 @@
       </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH1134)</t>
+          <t>IF$shsm:C&amp;O-1980:CO-3-dwarf(IH1134)</t>
         </is>
       </c>
       <c r="H137" t="inlineStr">
@@ -11914,7 +11914,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Head 36RA T G</t>
+          <t>Head 36RA T R</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -11929,7 +11929,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/135; packed 135 (node 1 sig 3); was S1-1 G</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/135; packed 135 (node 1 sig 3); was S1-1 G</t>
         </is>
       </c>
     </row>
@@ -11994,7 +11994,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Head 36RA T R</t>
+          <t>Head 36RA T G</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -12009,7 +12009,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/135; packed 135 (node 1 sig 3); was S1-1 R</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/135; packed 135 (node 1 sig 3); was S1-1 R</t>
         </is>
       </c>
     </row>
@@ -12034,7 +12034,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Head 36RA B G</t>
+          <t>Head 36RA B R</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -12049,7 +12049,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/136; packed 136 (node 1 sig 4); was S1-2 G</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/136; packed 136 (node 1 sig 4); was S1-2 G</t>
         </is>
       </c>
     </row>
@@ -12114,7 +12114,7 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Head 36RA B R</t>
+          <t>Head 36RA B G</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -12129,7 +12129,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/136; packed 136 (node 1 sig 4); was S1-2 R</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/136; packed 136 (node 1 sig 4); was S1-2 R</t>
         </is>
       </c>
     </row>
@@ -12154,7 +12154,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Head 38LA R</t>
+          <t>Head 38LA G</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -12169,7 +12169,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/143; packed 143 (node 1 sig 11)</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/143; packed 143 (node 1 sig 11)</t>
         </is>
       </c>
     </row>
@@ -12234,7 +12234,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Head 36RB T G</t>
+          <t>Head 36RB T R</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -12249,7 +12249,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/132; packed 132 (node 1 sig 0); was S1-3 G</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/132; packed 132 (node 1 sig 0); was S1-3 G</t>
         </is>
       </c>
     </row>
@@ -12314,7 +12314,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Head 36RB T R</t>
+          <t>Head 36RB T G</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -12329,7 +12329,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/132; packed 132 (node 1 sig 0); was S1-3 R</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/132; packed 132 (node 1 sig 0); was S1-3 R</t>
         </is>
       </c>
     </row>
@@ -12354,7 +12354,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Head 36RB B G</t>
+          <t>Head 36RB B R</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -12369,7 +12369,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/133; packed 133 (node 1 sig 1); was S1-4 G</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/133; packed 133 (node 1 sig 1); was S1-4 G</t>
         </is>
       </c>
     </row>
@@ -12434,7 +12434,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Head 36RB B R</t>
+          <t>Head 36RB B G</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -12449,7 +12449,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/133; packed 133 (node 1 sig 1); was S1-4 R</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/133; packed 133 (node 1 sig 1); was S1-4 R</t>
         </is>
       </c>
     </row>
@@ -12474,7 +12474,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Head 38LA G</t>
+          <t>Head 38LA R</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -12489,7 +12489,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/143; packed 143 (node 1 sig 11)</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/143; packed 143 (node 1 sig 11)</t>
         </is>
       </c>
     </row>
@@ -12874,7 +12874,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Head 34L T G</t>
+          <t>Head 34L T R</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -12889,7 +12889,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1232; packed 1232 (node 12 sig 0); was S2-1 G</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1232; packed 1232 (node 12 sig 0); was S2-1 G</t>
         </is>
       </c>
     </row>
@@ -12954,7 +12954,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Head 34L T R</t>
+          <t>Head 34L T G</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -12969,7 +12969,7 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1232; packed 1232 (node 12 sig 0); was S2-1 R</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1232; packed 1232 (node 12 sig 0); was S2-1 R</t>
         </is>
       </c>
     </row>
@@ -12994,7 +12994,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Head 34L B G</t>
+          <t>Head 34L B R</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -13009,7 +13009,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1233; packed 1233 (node 12 sig 1); was S2-2 G</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1233; packed 1233 (node 12 sig 1); was S2-2 G</t>
         </is>
       </c>
     </row>
@@ -13074,7 +13074,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Head 34L B R</t>
+          <t>Head 34L B G</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -13089,7 +13089,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1233; packed 1233 (node 12 sig 1); was S2-2 R</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1233; packed 1233 (node 12 sig 1); was S2-2 R</t>
         </is>
       </c>
     </row>
@@ -13114,7 +13114,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Head 32R G</t>
+          <t>Head 32R R</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -13129,7 +13129,7 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1234; packed 1234 (node 12 sig 2); was S2-8 Y</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1234; packed 1234 (node 12 sig 2); was S2-8 Y</t>
         </is>
       </c>
     </row>
@@ -13194,7 +13194,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Head 34R T G</t>
+          <t>Head 34R T R</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -13209,7 +13209,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1235; packed 1235 (node 12 sig 3); was S2-9 G</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1235; packed 1235 (node 12 sig 3); was S2-9 G</t>
         </is>
       </c>
     </row>
@@ -13274,7 +13274,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Head 34R T R</t>
+          <t>Head 34R T G</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -13289,7 +13289,7 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1235; packed 1235 (node 12 sig 3); was S2-9 Y</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1235; packed 1235 (node 12 sig 3); was S2-9 Y</t>
         </is>
       </c>
     </row>
@@ -13314,7 +13314,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Head 34R B G</t>
+          <t>Head 34R B R</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -13329,7 +13329,7 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1236; packed 1236 (node 12 sig 4); was S2-4 G</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1236; packed 1236 (node 12 sig 4); was S2-4 G</t>
         </is>
       </c>
     </row>
@@ -13394,7 +13394,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Head 34R B R</t>
+          <t>Head 34R B G</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -13409,7 +13409,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1236; packed 1236 (node 12 sig 4); was S2-4 R</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1236; packed 1236 (node 12 sig 4); was S2-4 R</t>
         </is>
       </c>
     </row>
@@ -13434,7 +13434,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Head 32R R</t>
+          <t>Head 32R G</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -13449,7 +13449,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1234; packed 1234 (node 12 sig 2); was S2-8 G</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1234; packed 1234 (node 12 sig 2); was S2-8 G</t>
         </is>
       </c>
     </row>
@@ -13514,7 +13514,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Head 24RA T G</t>
+          <t>Head 24RA T R</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
@@ -13529,7 +13529,7 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/232; packed 232 (node 2 sig 0)</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/232; packed 232 (node 2 sig 0)</t>
         </is>
       </c>
     </row>
@@ -13594,7 +13594,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Head 24RA T R</t>
+          <t>Head 24RA T G</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -13609,7 +13609,7 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/232; packed 232 (node 2 sig 0)</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/232; packed 232 (node 2 sig 0)</t>
         </is>
       </c>
     </row>
@@ -13634,7 +13634,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Head 24RA B G</t>
+          <t>Head 24RA B R</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -13649,7 +13649,7 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/238; packed 238 (node 2 sig 6)</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/238; packed 238 (node 2 sig 6)</t>
         </is>
       </c>
     </row>
@@ -13714,7 +13714,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Head 24RA B R</t>
+          <t>Head 24RA B G</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -13729,7 +13729,7 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/238; packed 238 (node 2 sig 6)</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/238; packed 238 (node 2 sig 6)</t>
         </is>
       </c>
     </row>
@@ -13824,7 +13824,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Head 24L T G</t>
+          <t>Head 24L T R</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -13839,7 +13839,7 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/233; packed 233 (node 2 sig 1); was S2-5 G</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/233; packed 233 (node 2 sig 1); was S2-5 G</t>
         </is>
       </c>
     </row>
@@ -13904,7 +13904,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Head 24L T R</t>
+          <t>Head 24L T G</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -13919,7 +13919,7 @@
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/233; packed 233 (node 2 sig 1); was S2-5 R</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/233; packed 233 (node 2 sig 1); was S2-5 R</t>
         </is>
       </c>
     </row>
@@ -13944,7 +13944,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Head 24L B G</t>
+          <t>Head 24L B R</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -13959,7 +13959,7 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/239; packed 239 (node 2 sig 7); was S2-3 G</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/239; packed 239 (node 2 sig 7); was S2-3 G</t>
         </is>
       </c>
     </row>
@@ -14024,7 +14024,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Head 24L B R</t>
+          <t>Head 24L B G</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -14039,7 +14039,7 @@
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/239; packed 239 (node 2 sig 7); was S2-3 R</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/239; packed 239 (node 2 sig 7); was S2-3 R</t>
         </is>
       </c>
     </row>
@@ -14279,7 +14279,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Head 24RB G</t>
+          <t>Head 24RB R</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -14294,7 +14294,7 @@
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/234; packed 234 (node 2 sig 2)</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/234; packed 234 (node 2 sig 2)</t>
         </is>
       </c>
     </row>
@@ -14359,7 +14359,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Head 24RB R</t>
+          <t>Head 24RB G</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -14374,7 +14374,7 @@
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/234; packed 234 (node 2 sig 2)</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/234; packed 234 (node 2 sig 2)</t>
         </is>
       </c>
     </row>
@@ -14969,7 +14969,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Head 8RA T G</t>
+          <t>Head 8RA T R</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -14984,7 +14984,7 @@
       </c>
       <c r="H90" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1332; packed 1332 (node 13 sig 0); was S3-10 G</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1332; packed 1332 (node 13 sig 0); was S3-10 G</t>
         </is>
       </c>
     </row>
@@ -15049,7 +15049,7 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Head 8RA T R</t>
+          <t>Head 8RA T G</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
@@ -15064,7 +15064,7 @@
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1332; packed 1332 (node 13 sig 0); was S3-10 R</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1332; packed 1332 (node 13 sig 0); was S3-10 R</t>
         </is>
       </c>
     </row>
@@ -15089,7 +15089,7 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Head 8RA B G</t>
+          <t>Head 8RA B R</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
@@ -15104,7 +15104,7 @@
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1333; packed 1333 (node 13 sig 1); was S3-12 G</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1333; packed 1333 (node 13 sig 1); was S3-12 G</t>
         </is>
       </c>
     </row>
@@ -15169,7 +15169,7 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Head 8RA B R</t>
+          <t>Head 8RA B G</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
@@ -15184,7 +15184,7 @@
       </c>
       <c r="H95" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1333; packed 1333 (node 13 sig 1); was S3-12 Y</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1333; packed 1333 (node 13 sig 1); was S3-12 Y</t>
         </is>
       </c>
     </row>
@@ -15279,7 +15279,7 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Head 8LA T G</t>
+          <t>Head 8LA T R</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
@@ -15294,7 +15294,7 @@
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1337; packed 1337 (node 13 sig 5); was S3-4 G</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1337; packed 1337 (node 13 sig 5); was S3-4 G</t>
         </is>
       </c>
     </row>
@@ -15359,7 +15359,7 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Head 8LA T R</t>
+          <t>Head 8LA T G</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
@@ -15374,7 +15374,7 @@
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1337; packed 1337 (node 13 sig 5); was S3-4 R</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1337; packed 1337 (node 13 sig 5); was S3-4 R</t>
         </is>
       </c>
     </row>
@@ -15399,7 +15399,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Head 8LA B G</t>
+          <t>Head 8LA B R</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
@@ -15414,7 +15414,7 @@
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1338; packed 1338 (node 13 sig 6); was S3-5 G</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1338; packed 1338 (node 13 sig 6); was S3-5 G</t>
         </is>
       </c>
     </row>
@@ -15479,7 +15479,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Head 8LA B R</t>
+          <t>Head 8LA B G</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -15494,7 +15494,7 @@
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1338; packed 1338 (node 13 sig 6); was S3-5 R</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1338; packed 1338 (node 13 sig 6); was S3-5 R</t>
         </is>
       </c>
     </row>
@@ -15519,7 +15519,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Head 8LB G</t>
+          <t>Head 8LB R</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
@@ -15534,7 +15534,7 @@
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1334; packed 1334 (node 13 sig 2); was S3-14 Y</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1334; packed 1334 (node 13 sig 2); was S3-14 Y</t>
         </is>
       </c>
     </row>
@@ -15919,7 +15919,7 @@
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Head 6LB T G</t>
+          <t>Head 6LB T R</t>
         </is>
       </c>
       <c r="F114" t="inlineStr">
@@ -15934,7 +15934,7 @@
       </c>
       <c r="H114" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/432; packed 432 (node 4 sig 0); was S3-1 G</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/432; packed 432 (node 4 sig 0); was S3-1 G</t>
         </is>
       </c>
     </row>
@@ -15999,7 +15999,7 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Head 6LB T R</t>
+          <t>Head 6LB T G</t>
         </is>
       </c>
       <c r="F116" t="inlineStr">
@@ -16014,7 +16014,7 @@
       </c>
       <c r="H116" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/432; packed 432 (node 4 sig 0); was S3-1 R</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/432; packed 432 (node 4 sig 0); was S3-1 R</t>
         </is>
       </c>
     </row>
@@ -16039,7 +16039,7 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>Head 6LB B G</t>
+          <t>Head 6LB B R</t>
         </is>
       </c>
       <c r="F117" t="inlineStr">
@@ -16054,7 +16054,7 @@
       </c>
       <c r="H117" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/433; packed 433 (node 4 sig 1); was S3-13 G</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/433; packed 433 (node 4 sig 1); was S3-13 G</t>
         </is>
       </c>
     </row>
@@ -16119,7 +16119,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>Head 6LB B R</t>
+          <t>Head 6LB B G</t>
         </is>
       </c>
       <c r="F119" t="inlineStr">
@@ -16134,7 +16134,7 @@
       </c>
       <c r="H119" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/433; packed 433 (node 4 sig 1); was S3-13 Y</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/433; packed 433 (node 4 sig 1); was S3-13 Y</t>
         </is>
       </c>
     </row>
@@ -16159,7 +16159,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Head 6LA G</t>
+          <t>Head 6LA R</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -16174,7 +16174,7 @@
       </c>
       <c r="H120" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/434; packed 434 (node 4 sig 2)</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/434; packed 434 (node 4 sig 2)</t>
         </is>
       </c>
     </row>
@@ -16239,7 +16239,7 @@
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>Head 2L T G</t>
+          <t>Head 2L T R</t>
         </is>
       </c>
       <c r="F122" t="inlineStr">
@@ -16254,7 +16254,7 @@
       </c>
       <c r="H122" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/438; packed 438 (node 4 sig 6); was S3-2 G</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/438; packed 438 (node 4 sig 6); was S3-2 G</t>
         </is>
       </c>
     </row>
@@ -16319,7 +16319,7 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>Head 2L T R</t>
+          <t>Head 2L T G</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
@@ -16334,7 +16334,7 @@
       </c>
       <c r="H124" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/438; packed 438 (node 4 sig 6); was S3-2 R</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/438; packed 438 (node 4 sig 6); was S3-2 R</t>
         </is>
       </c>
     </row>
@@ -16359,7 +16359,7 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>Head 2L B G</t>
+          <t>Head 2L B R</t>
         </is>
       </c>
       <c r="F125" t="inlineStr">
@@ -16374,7 +16374,7 @@
       </c>
       <c r="H125" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/439; packed 439 (node 4 sig 7); was S3-3 G</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/439; packed 439 (node 4 sig 7); was S3-3 G</t>
         </is>
       </c>
     </row>
@@ -16439,7 +16439,7 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>Head 2L B R</t>
+          <t>Head 2L B G</t>
         </is>
       </c>
       <c r="F127" t="inlineStr">
@@ -16454,7 +16454,7 @@
       </c>
       <c r="H127" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/439; packed 439 (node 4 sig 7); was S3-3 R</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/439; packed 439 (node 4 sig 7); was S3-3 R</t>
         </is>
       </c>
     </row>
@@ -16479,7 +16479,7 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>Head 6LA R</t>
+          <t>Head 6LA G</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
@@ -16494,7 +16494,7 @@
       </c>
       <c r="H128" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/434; packed 434 (node 4 sig 2)</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/434; packed 434 (node 4 sig 2)</t>
         </is>
       </c>
     </row>
@@ -16849,7 +16849,7 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>Head 40LB T G</t>
+          <t>Head 40LB T R</t>
         </is>
       </c>
       <c r="F138" t="inlineStr">
@@ -16864,7 +16864,7 @@
       </c>
       <c r="H138" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1132; packed 1132 (node 11 sig 0); was S1-5 G</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1132; packed 1132 (node 11 sig 0); was S1-5 G</t>
         </is>
       </c>
     </row>
@@ -16929,7 +16929,7 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>Head 40LB T R</t>
+          <t>Head 40LB T G</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
@@ -16944,7 +16944,7 @@
       </c>
       <c r="H140" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1132; packed 1132 (node 11 sig 0); was S1-5 Y</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1132; packed 1132 (node 11 sig 0); was S1-5 Y</t>
         </is>
       </c>
     </row>
@@ -16969,7 +16969,7 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>Head 40LB B G</t>
+          <t>Head 40LB B R</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
@@ -16984,7 +16984,7 @@
       </c>
       <c r="H141" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1135; packed 1135 (node 11 sig 3); was S1-6 G</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1135; packed 1135 (node 11 sig 3); was S1-6 G</t>
         </is>
       </c>
     </row>
@@ -17049,7 +17049,7 @@
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>Head 40LB B R</t>
+          <t>Head 40LB B G</t>
         </is>
       </c>
       <c r="F143" t="inlineStr">
@@ -17064,7 +17064,7 @@
       </c>
       <c r="H143" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1135; packed 1135 (node 11 sig 3); was S1-6 Y</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1135; packed 1135 (node 11 sig 3); was S1-6 Y</t>
         </is>
       </c>
     </row>
@@ -17089,7 +17089,7 @@
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>Head 2035 R</t>
+          <t>Head 2035 G</t>
         </is>
       </c>
       <c r="F144" t="inlineStr">
@@ -17104,7 +17104,7 @@
       </c>
       <c r="H144" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1134; packed 1134 (node 11 sig 2)</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1134; packed 1134 (node 11 sig 2)</t>
         </is>
       </c>
     </row>
@@ -17169,7 +17169,7 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>Head 40LA G</t>
+          <t>Head 40LA R</t>
         </is>
       </c>
       <c r="F146" t="inlineStr">
@@ -17184,7 +17184,7 @@
       </c>
       <c r="H146" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1136; packed 1136 (node 11 sig 4); was S4-6 G</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1136; packed 1136 (node 11 sig 4); was S4-6 G</t>
         </is>
       </c>
     </row>
@@ -17249,7 +17249,7 @@
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>Head 40LA R</t>
+          <t>Head 40LA G</t>
         </is>
       </c>
       <c r="F148" t="inlineStr">
@@ -17264,7 +17264,7 @@
       </c>
       <c r="H148" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1136; packed 1136 (node 11 sig 4); was S4-6 Y</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1136; packed 1136 (node 11 sig 4); was S4-6 Y</t>
         </is>
       </c>
     </row>
@@ -17289,7 +17289,7 @@
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>Head 2036 G</t>
+          <t>Head 2036 R</t>
         </is>
       </c>
       <c r="F149" t="inlineStr">
@@ -17304,7 +17304,7 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1133; packed 1133 (node 11 sig 1); was S4-7 G</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1133; packed 1133 (node 11 sig 1); was S4-7 G</t>
         </is>
       </c>
     </row>
@@ -17369,7 +17369,7 @@
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>Head 2036 R</t>
+          <t>Head 2036 G</t>
         </is>
       </c>
       <c r="F151" t="inlineStr">
@@ -17384,7 +17384,7 @@
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1133; packed 1133 (node 11 sig 1); was S4-7 Y</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1133; packed 1133 (node 11 sig 1); was S4-7 Y</t>
         </is>
       </c>
     </row>
@@ -17409,7 +17409,7 @@
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>Head 2035 G</t>
+          <t>Head 2035 R</t>
         </is>
       </c>
       <c r="F152" t="inlineStr">
@@ -17424,7 +17424,7 @@
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1134; packed 1134 (node 11 sig 2)</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1134; packed 1134 (node 11 sig 2)</t>
         </is>
       </c>
     </row>
@@ -23239,7 +23239,7 @@
       </c>
       <c r="E306" t="inlineStr">
         <is>
-          <t>Head 38LB T G</t>
+          <t>Head 38LB T R</t>
         </is>
       </c>
       <c r="F306" t="inlineStr">
@@ -23254,7 +23254,7 @@
       </c>
       <c r="H306" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/139; packed 139 (node 1 sig 7)</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/139; packed 139 (node 1 sig 7)</t>
         </is>
       </c>
     </row>
@@ -23319,7 +23319,7 @@
       </c>
       <c r="E308" t="inlineStr">
         <is>
-          <t>Head 38LB T R</t>
+          <t>Head 38LB T G</t>
         </is>
       </c>
       <c r="F308" t="inlineStr">
@@ -23334,7 +23334,7 @@
       </c>
       <c r="H308" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/139; packed 139 (node 1 sig 7)</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/139; packed 139 (node 1 sig 7)</t>
         </is>
       </c>
     </row>
@@ -23359,7 +23359,7 @@
       </c>
       <c r="E309" t="inlineStr">
         <is>
-          <t>Head 38LB B G</t>
+          <t>Head 38LB B R</t>
         </is>
       </c>
       <c r="F309" t="inlineStr">
@@ -23374,7 +23374,7 @@
       </c>
       <c r="H309" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/140; packed 140 (node 1 sig 8)</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/140; packed 140 (node 1 sig 8)</t>
         </is>
       </c>
     </row>
@@ -23439,7 +23439,7 @@
       </c>
       <c r="E311" t="inlineStr">
         <is>
-          <t>Head 38LB B R</t>
+          <t>Head 38LB B G</t>
         </is>
       </c>
       <c r="F311" t="inlineStr">
@@ -23454,7 +23454,7 @@
       </c>
       <c r="H311" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/140; packed 140 (node 1 sig 8)</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/140; packed 140 (node 1 sig 8)</t>
         </is>
       </c>
     </row>
@@ -23539,7 +23539,7 @@
       </c>
       <c r="E314" t="inlineStr">
         <is>
-          <t>Head 4RA G</t>
+          <t>Head 4RA R</t>
         </is>
       </c>
       <c r="F314" t="inlineStr">
@@ -23554,7 +23554,7 @@
       </c>
       <c r="H314" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/436; packed 436 (node 4 sig 4)</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/436; packed 436 (node 4 sig 4)</t>
         </is>
       </c>
     </row>
@@ -23619,7 +23619,7 @@
       </c>
       <c r="E316" t="inlineStr">
         <is>
-          <t>Head 4RA R</t>
+          <t>Head 4RA G</t>
         </is>
       </c>
       <c r="F316" t="inlineStr">
@@ -23634,7 +23634,7 @@
       </c>
       <c r="H316" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/436; packed 436 (node 4 sig 4)</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/436; packed 436 (node 4 sig 4)</t>
         </is>
       </c>
     </row>
@@ -23659,7 +23659,7 @@
       </c>
       <c r="E317" t="inlineStr">
         <is>
-          <t>Head 4RB G</t>
+          <t>Head 4RB R</t>
         </is>
       </c>
       <c r="F317" t="inlineStr">
@@ -23674,7 +23674,7 @@
       </c>
       <c r="H317" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/437; packed 437 (node 4 sig 5)</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/437; packed 437 (node 4 sig 5)</t>
         </is>
       </c>
     </row>
@@ -23739,7 +23739,7 @@
       </c>
       <c r="E319" t="inlineStr">
         <is>
-          <t>Head 4RB R</t>
+          <t>Head 4RB G</t>
         </is>
       </c>
       <c r="F319" t="inlineStr">
@@ -23754,7 +23754,7 @@
       </c>
       <c r="H319" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/437; packed 437 (node 4 sig 5)</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/437; packed 437 (node 4 sig 5)</t>
         </is>
       </c>
     </row>
@@ -23839,7 +23839,7 @@
       </c>
       <c r="E322" t="inlineStr">
         <is>
-          <t>Head 8RB T G</t>
+          <t>Head 8RB T R</t>
         </is>
       </c>
       <c r="F322" t="inlineStr">
@@ -23854,7 +23854,7 @@
       </c>
       <c r="H322" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1335; packed 1335 (node 13 sig 3)</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1335; packed 1335 (node 13 sig 3)</t>
         </is>
       </c>
     </row>
@@ -23919,7 +23919,7 @@
       </c>
       <c r="E324" t="inlineStr">
         <is>
-          <t>Head 8RB T R</t>
+          <t>Head 8RB T G</t>
         </is>
       </c>
       <c r="F324" t="inlineStr">
@@ -23934,7 +23934,7 @@
       </c>
       <c r="H324" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1335; packed 1335 (node 13 sig 3)</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1335; packed 1335 (node 13 sig 3)</t>
         </is>
       </c>
     </row>
@@ -23959,7 +23959,7 @@
       </c>
       <c r="E325" t="inlineStr">
         <is>
-          <t>Head 8RB B G</t>
+          <t>Head 8RB B R</t>
         </is>
       </c>
       <c r="F325" t="inlineStr">
@@ -23974,7 +23974,7 @@
       </c>
       <c r="H325" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1336; packed 1336 (node 13 sig 4)</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1336; packed 1336 (node 13 sig 4)</t>
         </is>
       </c>
     </row>
@@ -24039,7 +24039,7 @@
       </c>
       <c r="E327" t="inlineStr">
         <is>
-          <t>Head 8RB B R</t>
+          <t>Head 8RB B G</t>
         </is>
       </c>
       <c r="F327" t="inlineStr">
@@ -24054,7 +24054,7 @@
       </c>
       <c r="H327" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1336; packed 1336 (node 13 sig 4)</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1336; packed 1336 (node 13 sig 4)</t>
         </is>
       </c>
     </row>
@@ -24079,7 +24079,7 @@
       </c>
       <c r="E328" t="inlineStr">
         <is>
-          <t>Head 8LB R</t>
+          <t>Head 8LB G</t>
         </is>
       </c>
       <c r="F328" t="inlineStr">
@@ -24094,7 +24094,7 @@
       </c>
       <c r="H328" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1334; packed 1334 (node 13 sig 2)</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1334; packed 1334 (node 13 sig 2)</t>
         </is>
       </c>
     </row>
@@ -29562,17 +29562,17 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
+          <t>C1-OU2-1</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>C1-OU2-2</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
           <t>C1-OU2-3</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>C1-OU2-2</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>C1-OU2-1</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -29654,17 +29654,17 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
+          <t>C11-OU3-4</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>C11-OU3-5</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
           <t>C11-OU3-6</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>C11-OU3-5</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>C11-OU3-4</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -29751,17 +29751,17 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
+          <t>C11-OU3-7</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>C11-OU3-8</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
           <t>C11-OU2-7</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>C11-OU3-8</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>C11-OU3-7</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -29930,17 +29930,17 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
+          <t>C2-OU2-1</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>C2-OU2-2</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
           <t>C2-OU2-3</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>C2-OU2-2</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>C2-OU2-1</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -30027,17 +30027,17 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
+          <t>C12-OU2-1</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>C12-OU2-2</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
           <t>C12-OU2-3</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>C12-OU2-2</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>C12-OU2-1</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
@@ -30141,17 +30141,17 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
+          <t>C12-OU2-7</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>C12-OU3-8</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
           <t>C12-OU3-7</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>C12-OU3-8</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>C12-OU2-7</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -30558,17 +30558,17 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
+          <t>C4-OU3-1</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>C4-OU3-2</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
           <t>C4-OU3-3</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>C4-OU3-2</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>C4-OU3-1</t>
         </is>
       </c>
     </row>
@@ -30677,17 +30677,17 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
+          <t>C4-OU2-7</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>C4-OU3-8</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
           <t>C4-OU3-7</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>C4-OU3-8</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>C4-OU2-7</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -31547,17 +31547,17 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
+          <t>C13-OU1-1</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>C13-OU1-2</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
           <t>C13-OU1-3</t>
-        </is>
-      </c>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>C13-OU1-2</t>
-        </is>
-      </c>
-      <c r="K35" t="inlineStr">
-        <is>
-          <t>C13-OU1-1</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">

</xml_diff>

<commit_message>
Commission Barn/EH turnout FB and move C13 motors to OU2.
Switch 7/11/13 are TWOSENSOR (Pi tables); Switch 7/9/11 motors sit on C13-OU2 with Digicon 8LA/8LB moved to OU3. Wiring inventory and Signal Manager plan updated.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/cats/data/LCOS_Layout_Inventory_v85_signal_ports.xlsx
+++ b/cats/data/LCOS_Layout_Inventory_v85_signal_ports.xlsx
@@ -2932,7 +2932,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>C13-OU2-1</t>
+          <t>C13-OU3-1</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -3004,7 +3004,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>C13-OU2-2</t>
+          <t>C13-OU3-2</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -3076,7 +3076,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>C13-OU2-3</t>
+          <t>C13-OU3-3</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -3148,7 +3148,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>C13-OU2-4</t>
+          <t>C13-OU3-4</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -3213,14 +3213,14 @@
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>LCOS Signal 6 UID 38; STOP/APPROACH/CLEAR; lamp R; was with 8LA T on OU2</t>
+          <t>LCOS Signal 6 UID 38; STOP/APPROACH/CLEAR; lamp R; was with 8LA T on OU3</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>C13-OU2-5</t>
+          <t>C13-OU3-5</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -3285,14 +3285,14 @@
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>LCOS Signal 6 UID 38; STOP/APPROACH/CLEAR; lamp Y; was with 8LA T on OU2</t>
+          <t>LCOS Signal 6 UID 38; STOP/APPROACH/CLEAR; lamp Y; was with 8LA T on OU3</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>C13-OU2-6</t>
+          <t>C13-OU3-6</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -3357,14 +3357,14 @@
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>LCOS Signal 6 UID 38; STOP/APPROACH/CLEAR; lamp G; was with 8LA T on OU2</t>
+          <t>LCOS Signal 6 UID 38; STOP/APPROACH/CLEAR; lamp G; was with 8LA T on OU3</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>C13-OU2-7</t>
+          <t>C13-OU3-7</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -3429,14 +3429,14 @@
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp R; was R/Y with 8LA; G spills to 8RB OU4</t>
+          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp R; was R/Y with 8LA on OU3; G spills to 8RB OU4</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>C13-OU2-8</t>
+          <t>C13-OU3-8</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -3501,7 +3501,7 @@
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp Y; was R/Y with 8LA; G spills to 8RB OU4</t>
+          <t>LCOS Signal 2 UID 34; STOP/APPROACH/CLEAR; lamp Y; was R/Y with 8LA on OU3; G spills to 8RB OU4</t>
         </is>
       </c>
     </row>
@@ -8800,7 +8800,7 @@
       </c>
       <c r="J122" t="inlineStr">
         <is>
-          <t>C13-OU2-1 C13-OU2-2 C13-OU2-3 C13-OU2-4 C13-OU2-5 C13-OU2-6</t>
+          <t>C13-OU3-1 C13-OU3-2 C13-OU3-3 C13-OU3-4 C13-OU3-5 C13-OU3-6</t>
         </is>
       </c>
     </row>
@@ -8852,7 +8852,7 @@
       </c>
       <c r="J123" t="inlineStr">
         <is>
-          <t>C13-OU2-7 C13-OU2-8 C13-OU4-7</t>
+          <t>C13-OU3-7 C13-OU3-8 C13-OU4-7</t>
         </is>
       </c>
     </row>
@@ -10725,6 +10725,11 @@
       <c r="M10" t="n">
         <v>3</v>
       </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>C13-OU2-1, C13-OU2-2, C13-OU2-3, C13-OU2-4, C13-OU2-5, C13-OU2-6</t>
+        </is>
+      </c>
       <c r="O10" t="inlineStr">
         <is>
           <t>Switch 7, Switch 11, Switch 9</t>
@@ -10772,7 +10777,7 @@
       </c>
       <c r="AB10" t="inlineStr">
         <is>
-          <t>8RA, 8LA, 8LB, 8RB</t>
+          <t>8RA, S3-4, S3-5, S3-14, 8LA, 8LB, 8RB</t>
         </is>
       </c>
       <c r="AD10" t="inlineStr">
@@ -15271,7 +15276,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>West - Lower (Barn right)</t>
+          <t>West - Lower (Barn)</t>
         </is>
       </c>
       <c r="D98" t="n">
@@ -15279,22 +15284,22 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Head 8LA T R</t>
+          <t>Switch 7 N</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>Searchlight Signal Head</t>
+          <t>Turnout Motor</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>5V</t>
+          <t>12V</t>
         </is>
       </c>
       <c r="H98" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1337; packed 1337 (node 13 sig 5); was S3-4 G</t>
+          <t>radio 13 | M2T1308 / Node: 13 Turnout: 0 | DCC 117 | ports 1,2</t>
         </is>
       </c>
     </row>
@@ -15311,7 +15316,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>West - Lower (Barn right)</t>
+          <t>West - Lower (Barn)</t>
         </is>
       </c>
       <c r="D99" t="n">
@@ -15319,22 +15324,22 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Head 8LA T Y</t>
+          <t>Switch 7 R</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>Searchlight Signal Head</t>
+          <t>Turnout Motor</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>5V</t>
+          <t>12V</t>
         </is>
       </c>
       <c r="H99" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp Y; MQTT track/signalhead/1337; packed 1337 (node 13 sig 5); was S3-4 Y</t>
+          <t>radio 13 | M2T1308 / Node: 13 Turnout: 0 | DCC 117 | ports 1,2</t>
         </is>
       </c>
     </row>
@@ -15351,7 +15356,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>West - Lower (Barn right)</t>
+          <t>West - Lower (Barn)</t>
         </is>
       </c>
       <c r="D100" t="n">
@@ -15359,22 +15364,22 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Head 8LA T G</t>
+          <t>Switch 11 N</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>Searchlight Signal Head</t>
+          <t>Turnout Motor</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>5V</t>
+          <t>12V</t>
         </is>
       </c>
       <c r="H100" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1337; packed 1337 (node 13 sig 5); was S3-4 R</t>
+          <t>radio 13 | M2T1309 / Node: 13 Turnout: 1 | DCC 118 | ports 3,4</t>
         </is>
       </c>
     </row>
@@ -15391,7 +15396,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>West - Lower (Barn right)</t>
+          <t>West - Lower (Barn)</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -15399,22 +15404,22 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Head 8LA B R</t>
+          <t>Switch 11 R</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>Searchlight Signal Head</t>
+          <t>Turnout Motor</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>5V</t>
+          <t>12V</t>
         </is>
       </c>
       <c r="H101" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1338; packed 1338 (node 13 sig 6); was S3-5 G</t>
+          <t>radio 13 | M2T1309 / Node: 13 Turnout: 1 | DCC 118 | ports 3,4</t>
         </is>
       </c>
     </row>
@@ -15431,7 +15436,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>West - Lower (Barn right)</t>
+          <t>West - Lower (Barn)</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -15439,22 +15444,22 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Head 8LA B Y</t>
+          <t>Switch 9 N</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>Searchlight Signal Head</t>
+          <t>Turnout Motor</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>5V</t>
+          <t>12V</t>
         </is>
       </c>
       <c r="H102" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp Y; MQTT track/signalhead/1338; packed 1338 (node 13 sig 6); was S3-5 Y</t>
+          <t>radio 13 | M2T1310 / Node: 13 Turnout: 2 | DCC 119 | ports 5,6</t>
         </is>
       </c>
     </row>
@@ -15471,7 +15476,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>West - Lower (Barn right)</t>
+          <t>West - Lower (Barn)</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -15479,22 +15484,22 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Head 8LA B G</t>
+          <t>Switch 9 R</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>Searchlight Signal Head</t>
+          <t>Turnout Motor</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>5V</t>
+          <t>12V</t>
         </is>
       </c>
       <c r="H103" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1338; packed 1338 (node 13 sig 6); was S3-5 R</t>
+          <t>radio 13 | M2T1310 / Node: 13 Turnout: 2 | DCC 119 | ports 5,6</t>
         </is>
       </c>
     </row>
@@ -15511,30 +15516,20 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>West - Lower (Barn right)</t>
+          <t>West - Lower (Barn)</t>
         </is>
       </c>
       <c r="D104" t="n">
         <v>7</v>
       </c>
-      <c r="E104" t="inlineStr">
-        <is>
-          <t>Head 8LB R</t>
-        </is>
-      </c>
-      <c r="F104" t="inlineStr">
-        <is>
-          <t>Searchlight Signal Head</t>
-        </is>
-      </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>5V</t>
+          <t>12V</t>
         </is>
       </c>
       <c r="H104" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1334; packed 1334 (node 13 sig 2); was S3-14 Y</t>
+          <t>spare (was leftover S3 RGB; motors use 1–6)</t>
         </is>
       </c>
     </row>
@@ -15551,30 +15546,20 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>West - Lower (Barn right)</t>
+          <t>West - Lower (Barn)</t>
         </is>
       </c>
       <c r="D105" t="n">
         <v>8</v>
       </c>
-      <c r="E105" t="inlineStr">
-        <is>
-          <t>Head 8LB Y</t>
-        </is>
-      </c>
-      <c r="F105" t="inlineStr">
-        <is>
-          <t>Searchlight Signal Head</t>
-        </is>
-      </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>5V</t>
+          <t>12V</t>
         </is>
       </c>
       <c r="H105" t="inlineStr">
         <is>
-          <t>HART Digicon STOP/APPROACH/CLEAR; lamp Y; MQTT track/signalhead/1334; packed 1334 (node 13 sig 2)</t>
+          <t>spare</t>
         </is>
       </c>
     </row>
@@ -22651,7 +22636,7 @@
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>West - Lower</t>
+          <t>West - Lower (Barn right)</t>
         </is>
       </c>
       <c r="D290" t="n">
@@ -22659,22 +22644,22 @@
       </c>
       <c r="E290" t="inlineStr">
         <is>
-          <t>Switch 7 N</t>
+          <t>Head 8LA T R</t>
         </is>
       </c>
       <c r="F290" t="inlineStr">
         <is>
-          <t>Turnout Motor</t>
+          <t>Searchlight Signal Head</t>
         </is>
       </c>
       <c r="G290" t="inlineStr">
         <is>
-          <t>12V</t>
+          <t>5V</t>
         </is>
       </c>
       <c r="H290" t="inlineStr">
         <is>
-          <t>radio addr 13 | M2T1308 / switch_id 13-8 / DCC 117 | TO6; TO8 shares motor (IT37) | ASSUMED on new C13-OU3 12V board — confirm physical board ID</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1337; packed 1337 (node 13 sig 5)</t>
         </is>
       </c>
     </row>
@@ -22691,7 +22676,7 @@
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>West - Lower</t>
+          <t>West - Lower (Barn right)</t>
         </is>
       </c>
       <c r="D291" t="n">
@@ -22699,22 +22684,22 @@
       </c>
       <c r="E291" t="inlineStr">
         <is>
-          <t>Switch 7 R</t>
+          <t>Head 8LA T Y</t>
         </is>
       </c>
       <c r="F291" t="inlineStr">
         <is>
-          <t>Turnout Motor</t>
+          <t>Searchlight Signal Head</t>
         </is>
       </c>
       <c r="G291" t="inlineStr">
         <is>
-          <t>12V</t>
+          <t>5V</t>
         </is>
       </c>
       <c r="H291" t="inlineStr">
         <is>
-          <t>radio addr 13 | M2T1308 / switch_id 13-8 / DCC 117 | TO6 | ASSUMED on new C13-OU3 12V board — confirm physical board ID</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp Y; MQTT track/signalhead/1337; packed 1337 (node 13 sig 5)</t>
         </is>
       </c>
     </row>
@@ -22731,7 +22716,7 @@
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>West - Lower</t>
+          <t>West - Lower (Barn right)</t>
         </is>
       </c>
       <c r="D292" t="n">
@@ -22739,22 +22724,22 @@
       </c>
       <c r="E292" t="inlineStr">
         <is>
-          <t>Switch 11 N</t>
+          <t>Head 8LA T G</t>
         </is>
       </c>
       <c r="F292" t="inlineStr">
         <is>
-          <t>Turnout Motor</t>
+          <t>Searchlight Signal Head</t>
         </is>
       </c>
       <c r="G292" t="inlineStr">
         <is>
-          <t>12V</t>
+          <t>5V</t>
         </is>
       </c>
       <c r="H292" t="inlineStr">
         <is>
-          <t>radio addr 13 | M2T1309 / switch_id 13-9 / DCC 118 | TO11 | ASSUMED on new C13-OU3 12V board — confirm physical board ID</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1337; packed 1337 (node 13 sig 5)</t>
         </is>
       </c>
     </row>
@@ -22771,7 +22756,7 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>West - Lower</t>
+          <t>West - Lower (Barn right)</t>
         </is>
       </c>
       <c r="D293" t="n">
@@ -22779,22 +22764,22 @@
       </c>
       <c r="E293" t="inlineStr">
         <is>
-          <t>Switch 11 R</t>
+          <t>Head 8LA B R</t>
         </is>
       </c>
       <c r="F293" t="inlineStr">
         <is>
-          <t>Turnout Motor</t>
+          <t>Searchlight Signal Head</t>
         </is>
       </c>
       <c r="G293" t="inlineStr">
         <is>
-          <t>12V</t>
+          <t>5V</t>
         </is>
       </c>
       <c r="H293" t="inlineStr">
         <is>
-          <t>radio addr 13 | M2T1309 / switch_id 13-9 / DCC 118 | TO11 | ASSUMED on new C13-OU3 12V board — confirm physical board ID</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1338; packed 1338 (node 13 sig 6)</t>
         </is>
       </c>
     </row>
@@ -22811,7 +22796,7 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>West - Lower</t>
+          <t>West - Lower (Barn right)</t>
         </is>
       </c>
       <c r="D294" t="n">
@@ -22819,22 +22804,22 @@
       </c>
       <c r="E294" t="inlineStr">
         <is>
-          <t>Switch 9 N</t>
+          <t>Head 8LA B Y</t>
         </is>
       </c>
       <c r="F294" t="inlineStr">
         <is>
-          <t>Turnout Motor</t>
+          <t>Searchlight Signal Head</t>
         </is>
       </c>
       <c r="G294" t="inlineStr">
         <is>
-          <t>12V</t>
+          <t>5V</t>
         </is>
       </c>
       <c r="H294" t="inlineStr">
         <is>
-          <t>radio addr 13 | M2T1310 / switch_id 13-10 / DCC 119 | TO10 | ASSUMED on new C13-OU3 12V board — confirm physical board ID</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp Y; MQTT track/signalhead/1338; packed 1338 (node 13 sig 6)</t>
         </is>
       </c>
     </row>
@@ -22851,7 +22836,7 @@
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>West - Lower</t>
+          <t>West - Lower (Barn right)</t>
         </is>
       </c>
       <c r="D295" t="n">
@@ -22859,22 +22844,22 @@
       </c>
       <c r="E295" t="inlineStr">
         <is>
-          <t>Switch 9 R</t>
+          <t>Head 8LA B G</t>
         </is>
       </c>
       <c r="F295" t="inlineStr">
         <is>
-          <t>Turnout Motor</t>
+          <t>Searchlight Signal Head</t>
         </is>
       </c>
       <c r="G295" t="inlineStr">
         <is>
-          <t>12V</t>
+          <t>5V</t>
         </is>
       </c>
       <c r="H295" t="inlineStr">
         <is>
-          <t>radio addr 13 | M2T1310 / switch_id 13-10 / DCC 119 | TO10 | ASSUMED on new C13-OU3 12V board — confirm physical board ID</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp G; MQTT track/signalhead/1338; packed 1338 (node 13 sig 6)</t>
         </is>
       </c>
     </row>
@@ -22891,20 +22876,30 @@
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>West - Lower</t>
+          <t>West - Lower (Barn right)</t>
         </is>
       </c>
       <c r="D296" t="n">
         <v>7</v>
       </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>Head 8LB R</t>
+        </is>
+      </c>
+      <c r="F296" t="inlineStr">
+        <is>
+          <t>Searchlight Signal Head</t>
+        </is>
+      </c>
       <c r="G296" t="inlineStr">
         <is>
-          <t>12V</t>
+          <t>5V</t>
         </is>
       </c>
       <c r="H296" t="inlineStr">
         <is>
-          <t>free | C13-OU3 12V</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp R; MQTT track/signalhead/1334; packed 1334 (node 13 sig 2)</t>
         </is>
       </c>
     </row>
@@ -22921,20 +22916,30 @@
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>West - Lower</t>
+          <t>West - Lower (Barn right)</t>
         </is>
       </c>
       <c r="D297" t="n">
         <v>8</v>
       </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>Head 8LB Y</t>
+        </is>
+      </c>
+      <c r="F297" t="inlineStr">
+        <is>
+          <t>Searchlight Signal Head</t>
+        </is>
+      </c>
       <c r="G297" t="inlineStr">
         <is>
-          <t>12V</t>
+          <t>5V</t>
         </is>
       </c>
       <c r="H297" t="inlineStr">
         <is>
-          <t>free | C13-OU3 12V</t>
+          <t>HART Digicon STOP/APPROACH/CLEAR; lamp Y; MQTT track/signalhead/1334; packed 1334 (node 13 sig 2)</t>
         </is>
       </c>
     </row>
@@ -28545,7 +28550,7 @@
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>M2S1367 / Switch 13-1 FB N | ASSUMED on new C13-IN1 — confirm physical board ID</t>
+          <t>M2S1367 / Switch 13-1 FB N | commissioned 2026-09-08</t>
         </is>
       </c>
     </row>
@@ -28580,7 +28585,7 @@
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>M2S1368 / Switch 13-1 FB R | ASSUMED on new C13-IN1 — confirm physical board ID</t>
+          <t>M2S1368 / Switch 13-1 FB R | commissioned 2026-09-08</t>
         </is>
       </c>
     </row>
@@ -28615,7 +28620,7 @@
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>M2S1369 / Switch 13-2 FB N | ASSUMED on new C13-IN1 — confirm physical board ID</t>
+          <t>M2S1369 / Switch 13-2 FB N | commissioned 2026-09-08</t>
         </is>
       </c>
     </row>
@@ -28650,7 +28655,7 @@
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>M2S1370 / Switch 13-2 FB R | ASSUMED on new C13-IN1 — confirm physical board ID</t>
+          <t>M2S1370 / Switch 13-2 FB R | commissioned 2026-09-08</t>
         </is>
       </c>
     </row>
@@ -28685,7 +28690,7 @@
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>M2S1371 / Switch 13-3 FB N | ASSUMED on new C13-IN1 — confirm physical board ID</t>
+          <t>M2S1371 / Switch 13-3 FB N | commissioned 2026-09-08</t>
         </is>
       </c>
     </row>
@@ -28720,7 +28725,7 @@
       </c>
       <c r="G151" t="inlineStr">
         <is>
-          <t>M2S1372 / Switch 13-3 FB R | ASSUMED on new C13-IN1 — confirm physical board ID</t>
+          <t>M2S1372 / Switch 13-3 FB R | commissioned 2026-09-08</t>
         </is>
       </c>
     </row>
@@ -28755,7 +28760,7 @@
       </c>
       <c r="G152" t="inlineStr">
         <is>
-          <t>ASSUMED on new C13-IN2 — confirm</t>
+          <t>local button; confirm silk</t>
         </is>
       </c>
     </row>
@@ -28790,7 +28795,7 @@
       </c>
       <c r="G153" t="inlineStr">
         <is>
-          <t>ASSUMED on new C13-IN2 — confirm</t>
+          <t>local button; confirm silk</t>
         </is>
       </c>
     </row>
@@ -28825,7 +28830,7 @@
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>ASSUMED on new C13-IN2 — confirm</t>
+          <t>local button; confirm silk</t>
         </is>
       </c>
     </row>
@@ -31565,9 +31570,39 @@
           <t>8LA</t>
         </is>
       </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>C13-OU3-1</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>C13-OU3-2</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>C13-OU3-3</t>
+        </is>
+      </c>
       <c r="P35" t="inlineStr">
         <is>
           <t>8LB / 8RB</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>C13-OU3-7</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>C13-OU3-8</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>C13-OU4-7</t>
         </is>
       </c>
     </row>

</xml_diff>